<commit_message>
Startaufbau durchnummeriert, Eckdaten entfernt
</commit_message>
<xml_diff>
--- a/data/startaufbau.xlsx
+++ b/data/startaufbau.xlsx
@@ -1162,7 +1162,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1304,7 +1304,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1375,7 +1375,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1450,7 +1450,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1521,7 +1521,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1663,7 +1663,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1734,7 +1734,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1805,7 +1805,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1947,7 +1947,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>

</xml_diff>